<commit_message>
fiox spawn & monster move
</commit_message>
<xml_diff>
--- a/eoe/Assets/Excels/MonsterConfig.xlsx
+++ b/eoe/Assets/Excels/MonsterConfig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Idle-rpg\eoe\Assets\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAD807A-681D-466C-9CA0-63F8AD034C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0044399-B7A1-4F46-B8BC-2EF185EE4B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>id</t>
   </si>
@@ -49,12 +49,6 @@
   </si>
   <si>
     <t>prefabName</t>
-  </si>
-  <si>
-    <t>deathVfxName</t>
-  </si>
-  <si>
-    <t>deathAudioClipName</t>
   </si>
   <si>
     <t>attackRange</t>
@@ -378,7 +372,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.6328125" style="1" customWidth="1"/>
@@ -387,12 +381,10 @@
     <col min="8" max="8" width="17.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.6328125" style="1" customWidth="1"/>
     <col min="10" max="10" width="23.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.26953125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="19.90625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="15.6328125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.6328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -415,25 +407,19 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>1001</v>
       </c>
@@ -464,7 +450,7 @@
       <c r="J2" s="1">
         <v>1</v>
       </c>
-      <c r="M2" s="1">
+      <c r="K2" s="1">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add elite and boss monster skills
</commit_message>
<xml_diff>
--- a/eoe/Assets/Excels/MonsterConfig.xlsx
+++ b/eoe/Assets/Excels/MonsterConfig.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.5" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15.63" customWidth="1" style="2" min="1" max="1"/>
@@ -412,6 +412,16 @@
           <t>gold</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="16.5" customHeight="1" s="3">
       <c r="A2" s="2" t="n">
@@ -449,79 +459,109 @@
       <c r="K2" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>1002</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>monster.1002</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="0" t="n">
         <v>0.9</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="0" t="n">
         <v>0.8</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="0" t="n">
         <v>7</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>[{"skillId":2002,"cooldown":4.0,"damageMultiplier":1.5}]</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="0" t="n">
         <v>1003</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>monster.1003</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="0" t="n">
         <v>2.5</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="0" t="n">
         <v>10</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>[{"skillId":2005,"cooldown":5.0,"damageMultiplier":2.0},{"skillId":2006,"cooldown":7.0,"damageMultiplier":1.25},{"skillId":2007,"cooldown":6.0,"damageMultiplier":1.0}]</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add second hero and one-hit-per-second monsters
</commit_message>
<xml_diff>
--- a/eoe/Assets/Excels/MonsterConfig.xlsx
+++ b/eoe/Assets/Excels/MonsterConfig.xlsx
@@ -394,7 +394,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>attackCooldown</t>
+          <t>damageCooldown</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
@@ -412,12 +412,12 @@
           <t>gold</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="0" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="0" t="inlineStr">
         <is>
           <t>skills</t>
         </is>
@@ -448,7 +448,7 @@
         <v>0.5</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>2</v>
@@ -459,12 +459,12 @@
       <c r="K2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="0" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="0" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
@@ -495,7 +495,7 @@
         <v>0.5</v>
       </c>
       <c r="H3" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3" s="0" t="n">
         <v>2</v>
@@ -506,12 +506,12 @@
       <c r="K3" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="0" t="inlineStr">
         <is>
           <t>Elite</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" s="0" t="inlineStr">
         <is>
           <t>[{"skillId":2002,"cooldown":4.0,"damageMultiplier":1.5}]</t>
         </is>
@@ -542,7 +542,7 @@
         <v>0.7</v>
       </c>
       <c r="H4" s="0" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="I4" s="0" t="n">
         <v>2</v>
@@ -553,12 +553,12 @@
       <c r="K4" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="0" t="inlineStr">
         <is>
           <t>Boss</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" s="0" t="inlineStr">
         <is>
           <t>[{"skillId":2005,"cooldown":5.0,"damageMultiplier":2.0},{"skillId":2006,"cooldown":7.0,"damageMultiplier":1.25},{"skillId":2007,"cooldown":6.0,"damageMultiplier":1.0}]</t>
         </is>

</xml_diff>

<commit_message>
feat: add post-wave upgrades and status rules
</commit_message>
<xml_diff>
--- a/eoe/Assets/Excels/MonsterConfig.xlsx
+++ b/eoe/Assets/Excels/MonsterConfig.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.5" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15.63" customWidth="1" style="2" min="1" max="1"/>
@@ -422,6 +422,11 @@
           <t>skills</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>statusResistances</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="16.5" customHeight="1" s="3">
       <c r="A2" s="2" t="n">
@@ -469,6 +474,11 @@
           <t>[]</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>[{"type":1,"resistance":0.0},{"type":2,"resistance":0.0},{"type":3,"resistance":0.0},{"type":4,"resistance":0.0}]</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="n">
@@ -516,6 +526,11 @@
           <t>[{"skillId":2002,"cooldown":4.0,"damageMultiplier":1.5}]</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>[{"type":1,"resistance":0.25},{"type":2,"resistance":0.2},{"type":3,"resistance":0.35},{"type":4,"resistance":0.25}]</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="n">
@@ -561,6 +576,11 @@
       <c r="M4" s="0" t="inlineStr">
         <is>
           <t>[{"skillId":2005,"cooldown":5.0,"damageMultiplier":2.0},{"skillId":2006,"cooldown":7.0,"damageMultiplier":1.25},{"skillId":2007,"cooldown":6.0,"damageMultiplier":1.0}]</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>[{"type":1,"resistance":0.5},{"type":2,"resistance":0.4},{"type":3,"resistance":0.6},{"type":4,"resistance":0.5}]</t>
         </is>
       </c>
     </row>

</xml_diff>